<commit_message>
update the excel sheet
</commit_message>
<xml_diff>
--- a/12624002.xlsx
+++ b/12624002.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c135914e813e79f/Desktop/python/776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="168" documentId="8_{2F929DCF-A852-4FE5-927A-37AC65437CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EFD341D-1911-44D8-A238-6E4323E52D83}"/>
+  <xr:revisionPtr revIDLastSave="218" documentId="8_{2F929DCF-A852-4FE5-927A-37AC65437CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE41E0AB-BDE0-4A07-9AAE-9703069D480E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1985,91 +1985,179 @@
       <c r="N27" s="17"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B28" s="14">
+        <v>600</v>
+      </c>
+      <c r="C28" s="14">
+        <v>90</v>
+      </c>
+      <c r="D28" s="14">
+        <v>45</v>
+      </c>
+      <c r="E28" s="14">
+        <v>30</v>
+      </c>
+      <c r="F28" s="14">
+        <v>350</v>
+      </c>
+      <c r="G28" s="14">
+        <v>7</v>
+      </c>
+      <c r="H28" s="14">
+        <v>250</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1365</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
+        <v>75</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>59</v>
+      </c>
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="A29" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B29" s="14">
+        <v>580</v>
+      </c>
+      <c r="C29" s="14">
+        <v>100</v>
+      </c>
+      <c r="D29" s="14">
+        <v>0</v>
+      </c>
+      <c r="E29" s="14">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14">
+        <v>200</v>
+      </c>
+      <c r="G29" s="14">
+        <v>4</v>
+      </c>
+      <c r="H29" s="14">
+        <v>420</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1300</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
+        <v>140</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N29" s="17"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+      <c r="A30" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B30" s="14">
+        <v>600</v>
+      </c>
+      <c r="C30" s="14">
+        <v>90</v>
+      </c>
+      <c r="D30" s="14">
+        <v>65</v>
+      </c>
+      <c r="E30" s="14">
+        <v>55</v>
+      </c>
+      <c r="F30" s="14">
+        <v>250</v>
+      </c>
+      <c r="G30" s="14">
+        <v>5</v>
+      </c>
+      <c r="H30" s="14">
+        <v>350</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1410</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
+        <v>30</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N30" s="17"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+      <c r="A31" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B31" s="14">
+        <v>650</v>
+      </c>
+      <c r="C31" s="14">
+        <v>0</v>
+      </c>
+      <c r="D31" s="14">
+        <v>75</v>
+      </c>
+      <c r="E31" s="14">
+        <v>0</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <v>420</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>1145</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
+        <v>295</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N31" s="17"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>